<commit_message>
Finish refresh test data
</commit_message>
<xml_diff>
--- a/java22 database design/Java22 HDoan Database Design.xlsx
+++ b/java22 database design/Java22 HDoan Database Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace-it\code\course-webapp\java22\3. Database\java22 database design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2F7FF45-3BB3-46C9-8894-3424C48CDF7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16539D8-FC84-4757-B2CA-0F389CB5BC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="878" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1776" yWindow="1776" windowWidth="17280" windowHeight="8880" tabRatio="878" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -881,7 +881,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="550">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="557">
   <si>
     <t>NhanVien</t>
   </si>
@@ -2368,9 +2368,6 @@
   </si>
   <si>
     <t>Mặt Hàng 1-4</t>
-  </si>
-  <si>
-    <t>Mặt Hàng 1-8</t>
   </si>
   <si>
     <t>Mặt Hàng 9-12</t>
@@ -2545,12 +2542,36 @@
   <si>
     <t>C09_PAYMENT_METHOD_TYPE</t>
   </si>
+  <si>
+    <t>Mặt Hàng 5-8</t>
+  </si>
+  <si>
+    <t>c1@gmail.com</t>
+  </si>
+  <si>
+    <t>c2@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$12$qogFuuGROcCYCIbCOjQPaeOMmPcqRUFazWTqYpCv9lq88kE35JmkC</t>
+  </si>
+  <si>
+    <t>secret_password</t>
+  </si>
+  <si>
+    <t>-- 5. Đơn hàng từ 13  --&gt; Giao hàng thất bại (trạng thái 1,2,3,4,6)</t>
+  </si>
+  <si>
+    <t>-- 4. Đơn hàng từ 11 - 12 --&gt; Hủy đơn hàng (trạng thái 1 và 7)</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2739,6 +2760,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -2829,10 +2858,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3021,6 +3051,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3049,7 +3082,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -5777,16 +5811,16 @@
     </row>
     <row r="72" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="73" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C73" s="72" t="s">
+      <c r="C73" s="73" t="s">
         <v>277</v>
       </c>
-      <c r="D73" s="72"/>
-      <c r="E73" s="72"/>
+      <c r="D73" s="73"/>
+      <c r="E73" s="73"/>
     </row>
     <row r="74" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C74" s="72"/>
-      <c r="D74" s="72"/>
-      <c r="E74" s="72"/>
+      <c r="C74" s="73"/>
+      <c r="D74" s="73"/>
+      <c r="E74" s="73"/>
     </row>
     <row r="75" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="76" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -5810,14 +5844,14 @@
     </row>
     <row r="78" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="79" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C79" s="72" t="s">
+      <c r="C79" s="73" t="s">
         <v>277</v>
       </c>
-      <c r="D79" s="72"/>
+      <c r="D79" s="73"/>
     </row>
     <row r="80" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C80" s="72"/>
-      <c r="D80" s="72"/>
+      <c r="C80" s="73"/>
+      <c r="D80" s="73"/>
     </row>
     <row r="81" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="82" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -5852,30 +5886,30 @@
       </c>
     </row>
     <row r="86" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C86" s="73" t="s">
+      <c r="C86" s="74" t="s">
         <v>283</v>
       </c>
-      <c r="D86" s="72"/>
-      <c r="E86" s="72"/>
-      <c r="F86" s="72"/>
+      <c r="D86" s="73"/>
+      <c r="E86" s="73"/>
+      <c r="F86" s="73"/>
     </row>
     <row r="87" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C87" s="72"/>
-      <c r="D87" s="72"/>
-      <c r="E87" s="72"/>
-      <c r="F87" s="72"/>
+      <c r="C87" s="73"/>
+      <c r="D87" s="73"/>
+      <c r="E87" s="73"/>
+      <c r="F87" s="73"/>
     </row>
     <row r="88" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C88" s="72"/>
-      <c r="D88" s="72"/>
-      <c r="E88" s="72"/>
-      <c r="F88" s="72"/>
+      <c r="C88" s="73"/>
+      <c r="D88" s="73"/>
+      <c r="E88" s="73"/>
+      <c r="F88" s="73"/>
     </row>
     <row r="89" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C89" s="72"/>
-      <c r="D89" s="72"/>
-      <c r="E89" s="72"/>
-      <c r="F89" s="72"/>
+      <c r="C89" s="73"/>
+      <c r="D89" s="73"/>
+      <c r="E89" s="73"/>
+      <c r="F89" s="73"/>
     </row>
     <row r="90" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="91" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -5892,18 +5926,18 @@
       </c>
     </row>
     <row r="93" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="74" t="s">
+      <c r="B93" s="75" t="s">
         <v>280</v>
       </c>
-      <c r="C93" s="74"/>
+      <c r="C93" s="75"/>
     </row>
     <row r="94" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B94" s="72"/>
-      <c r="C94" s="72"/>
+      <c r="B94" s="73"/>
+      <c r="C94" s="73"/>
     </row>
     <row r="95" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B95" s="72"/>
-      <c r="C95" s="72"/>
+      <c r="B95" s="73"/>
+      <c r="C95" s="73"/>
     </row>
     <row r="96" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="97" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -5926,11 +5960,11 @@
       </c>
     </row>
     <row r="99" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="71" t="s">
+      <c r="B99" s="72" t="s">
         <v>281</v>
       </c>
-      <c r="C99" s="71"/>
-      <c r="D99" s="71"/>
+      <c r="C99" s="72"/>
+      <c r="D99" s="72"/>
       <c r="F99" s="14" t="s">
         <v>112</v>
       </c>
@@ -5945,14 +5979,14 @@
       </c>
     </row>
     <row r="100" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="71"/>
-      <c r="C100" s="71"/>
-      <c r="D100" s="71"/>
+      <c r="B100" s="72"/>
+      <c r="C100" s="72"/>
+      <c r="D100" s="72"/>
     </row>
     <row r="101" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B101" s="71"/>
-      <c r="C101" s="71"/>
-      <c r="D101" s="71"/>
+      <c r="B101" s="72"/>
+      <c r="C101" s="72"/>
+      <c r="D101" s="72"/>
       <c r="F101" s="31" t="s">
         <v>297</v>
       </c>
@@ -5960,7 +5994,7 @@
         <v>253</v>
       </c>
       <c r="I101" s="27" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="102" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -7641,15 +7675,15 @@
       <c r="K16" s="24"/>
     </row>
     <row r="17" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="66" t="s">
+      <c r="B17" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="66"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="68"/>
+      <c r="C17" s="67"/>
+      <c r="D17" s="67"/>
+      <c r="E17" s="67"/>
+      <c r="G17" s="69"/>
+      <c r="H17" s="69"/>
+      <c r="I17" s="69"/>
     </row>
     <row r="18" spans="2:11" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="10" t="s">
@@ -7661,12 +7695,12 @@
       <c r="I18" s="19"/>
     </row>
     <row r="19" spans="2:11" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="66" t="s">
+      <c r="B19" s="67" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="67"/>
-      <c r="D19" s="67"/>
-      <c r="E19" s="67"/>
+      <c r="C19" s="68"/>
+      <c r="D19" s="68"/>
+      <c r="E19" s="68"/>
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
     </row>
@@ -7678,12 +7712,12 @@
       <c r="K20" s="17"/>
     </row>
     <row r="21" spans="2:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="66" t="s">
+      <c r="B21" s="67" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="69"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="69"/>
+      <c r="C21" s="70"/>
+      <c r="D21" s="70"/>
+      <c r="E21" s="70"/>
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
@@ -7698,32 +7732,32 @@
       <c r="K22" s="20"/>
     </row>
     <row r="23" spans="2:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="67" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="66"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
+      <c r="C23" s="67"/>
+      <c r="D23" s="67"/>
+      <c r="E23" s="67"/>
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
     </row>
     <row r="24" spans="2:11" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="66" t="s">
+      <c r="B24" s="67" t="s">
         <v>338</v>
       </c>
-      <c r="C24" s="67"/>
-      <c r="D24" s="67"/>
-      <c r="E24" s="67"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
       <c r="J24" s="7"/>
       <c r="K24" s="7"/>
     </row>
     <row r="25" spans="2:11" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="66" t="s">
+      <c r="B25" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="67"/>
-      <c r="D25" s="67"/>
-      <c r="E25" s="67"/>
+      <c r="C25" s="68"/>
+      <c r="D25" s="68"/>
+      <c r="E25" s="68"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
       <c r="H25" s="4"/>
@@ -7957,16 +7991,16 @@
     </row>
     <row r="3" spans="2:21" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -7978,7 +8012,7 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
       <c r="O3" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="6"/>
@@ -8058,7 +8092,7 @@
         <v>443</v>
       </c>
       <c r="I5" s="38" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="J5" s="38" t="s">
         <v>462</v>
@@ -8067,7 +8101,7 @@
         <v>448</v>
       </c>
       <c r="L5" s="38" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="M5" s="38" t="s">
         <v>455</v>
@@ -8119,7 +8153,7 @@
         <v>449</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>456</v>
@@ -8175,7 +8209,7 @@
         <v>473</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="Q7" s="3"/>
       <c r="R7" s="18"/>
@@ -8208,10 +8242,10 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
       <c r="O8" s="3" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="18"/>
@@ -8230,11 +8264,11 @@
         <v>424</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H9" s="60"/>
       <c r="I9" s="3" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3" t="s">
@@ -8245,7 +8279,7 @@
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
       <c r="P9" s="3" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
@@ -8276,7 +8310,7 @@
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="Q10" s="18"/>
       <c r="R10" s="3"/>
@@ -8395,18 +8429,18 @@
       </c>
     </row>
     <row r="17" spans="4:18" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="66" t="s">
+      <c r="D17" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="66"/>
-      <c r="F17" s="66"/>
-      <c r="G17" s="66"/>
-      <c r="H17" s="66"/>
-      <c r="I17" s="66"/>
-      <c r="J17" s="66"/>
-      <c r="K17" s="68"/>
-      <c r="L17" s="68"/>
-      <c r="M17" s="68"/>
+      <c r="E17" s="67"/>
+      <c r="F17" s="67"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="67"/>
+      <c r="I17" s="67"/>
+      <c r="J17" s="67"/>
+      <c r="K17" s="69"/>
+      <c r="L17" s="69"/>
+      <c r="M17" s="69"/>
       <c r="O17" s="1">
         <v>1</v>
       </c>
@@ -8438,15 +8472,15 @@
       </c>
     </row>
     <row r="19" spans="4:18" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D19" s="66" t="s">
+      <c r="D19" s="67" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="67"/>
-      <c r="F19" s="67"/>
-      <c r="G19" s="67"/>
-      <c r="H19" s="67"/>
-      <c r="I19" s="67"/>
-      <c r="J19" s="67"/>
+      <c r="E19" s="68"/>
+      <c r="F19" s="68"/>
+      <c r="G19" s="68"/>
+      <c r="H19" s="68"/>
+      <c r="I19" s="68"/>
+      <c r="J19" s="68"/>
       <c r="N19" s="17"/>
       <c r="O19" s="17">
         <v>3</v>
@@ -8474,15 +8508,15 @@
       </c>
     </row>
     <row r="21" spans="4:18" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D21" s="66" t="s">
+      <c r="D21" s="67" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
-      <c r="G21" s="69"/>
-      <c r="H21" s="69"/>
-      <c r="I21" s="69"/>
-      <c r="J21" s="69"/>
+      <c r="E21" s="70"/>
+      <c r="F21" s="70"/>
+      <c r="G21" s="70"/>
+      <c r="H21" s="70"/>
+      <c r="I21" s="70"/>
+      <c r="J21" s="70"/>
       <c r="N21" s="17"/>
       <c r="O21" s="1">
         <v>5</v>
@@ -8516,15 +8550,15 @@
       </c>
     </row>
     <row r="23" spans="4:18" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D23" s="66" t="s">
+      <c r="D23" s="67" t="s">
         <v>50</v>
       </c>
-      <c r="E23" s="66"/>
-      <c r="F23" s="66"/>
-      <c r="G23" s="66"/>
-      <c r="H23" s="66"/>
-      <c r="I23" s="66"/>
-      <c r="J23" s="66"/>
+      <c r="E23" s="67"/>
+      <c r="F23" s="67"/>
+      <c r="G23" s="67"/>
+      <c r="H23" s="67"/>
+      <c r="I23" s="67"/>
+      <c r="J23" s="67"/>
       <c r="N23" s="7"/>
       <c r="O23" s="17">
         <v>7</v>
@@ -8537,15 +8571,15 @@
       </c>
     </row>
     <row r="24" spans="4:18" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D24" s="66" t="s">
+      <c r="D24" s="67" t="s">
         <v>338</v>
       </c>
-      <c r="E24" s="67"/>
-      <c r="F24" s="67"/>
-      <c r="G24" s="67"/>
-      <c r="H24" s="67"/>
-      <c r="I24" s="67"/>
-      <c r="J24" s="67"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="68"/>
+      <c r="J24" s="68"/>
       <c r="N24" s="7"/>
       <c r="O24" s="17">
         <v>8</v>
@@ -8558,15 +8592,15 @@
       </c>
     </row>
     <row r="25" spans="4:18" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D25" s="66" t="s">
+      <c r="D25" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="67"/>
-      <c r="F25" s="67"/>
-      <c r="G25" s="67"/>
-      <c r="H25" s="67"/>
-      <c r="I25" s="67"/>
-      <c r="J25" s="67"/>
+      <c r="E25" s="68"/>
+      <c r="F25" s="68"/>
+      <c r="G25" s="68"/>
+      <c r="H25" s="68"/>
+      <c r="I25" s="68"/>
+      <c r="J25" s="68"/>
       <c r="K25" s="15"/>
       <c r="L25" s="4"/>
       <c r="P25" s="15"/>
@@ -9187,7 +9221,7 @@
         <v>352</v>
       </c>
       <c r="E43" s="27" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="44" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9221,65 +9255,65 @@
         <v>1</v>
       </c>
       <c r="E45" s="28" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="F45" s="28" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G45" s="28" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="46" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="28"/>
       <c r="C46" s="28" t="s">
-        <v>493</v>
+        <v>549</v>
       </c>
       <c r="D46" s="28">
         <v>2</v>
       </c>
       <c r="E46" s="28" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="F46" s="28" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G46" s="28" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="47" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="28"/>
       <c r="C47" s="28" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="D47" s="28">
         <v>3</v>
       </c>
       <c r="E47" s="28"/>
       <c r="F47" s="28" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G47" s="28"/>
     </row>
     <row r="48" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="28"/>
       <c r="C48" s="28" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="D48" s="28">
         <v>4</v>
       </c>
       <c r="E48" s="28"/>
       <c r="F48" s="29" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G48" s="28"/>
     </row>
     <row r="49" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="28"/>
       <c r="C49" s="28" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="D49" s="28">
         <v>5</v>
@@ -9305,7 +9339,7 @@
         <v>473</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="53" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9476,34 +9510,34 @@
     </row>
     <row r="66" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="27" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="67" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C67" s="70" t="s">
-        <v>508</v>
-      </c>
-      <c r="D67" s="68"/>
-      <c r="E67" s="68"/>
-      <c r="F67" s="68"/>
+      <c r="C67" s="71" t="s">
+        <v>507</v>
+      </c>
+      <c r="D67" s="69"/>
+      <c r="E67" s="69"/>
+      <c r="F67" s="69"/>
     </row>
     <row r="68" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C68" s="68"/>
-      <c r="D68" s="68"/>
-      <c r="E68" s="68"/>
-      <c r="F68" s="68"/>
+      <c r="C68" s="69"/>
+      <c r="D68" s="69"/>
+      <c r="E68" s="69"/>
+      <c r="F68" s="69"/>
     </row>
     <row r="69" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C69" s="68"/>
-      <c r="D69" s="68"/>
-      <c r="E69" s="68"/>
-      <c r="F69" s="68"/>
+      <c r="C69" s="69"/>
+      <c r="D69" s="69"/>
+      <c r="E69" s="69"/>
+      <c r="F69" s="69"/>
     </row>
     <row r="70" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C70" s="68"/>
-      <c r="D70" s="68"/>
-      <c r="E70" s="68"/>
-      <c r="F70" s="68"/>
+      <c r="C70" s="69"/>
+      <c r="D70" s="69"/>
+      <c r="E70" s="69"/>
+      <c r="F70" s="69"/>
     </row>
     <row r="71" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9524,7 +9558,7 @@
         <v>1</v>
       </c>
       <c r="C74" s="28" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="75" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9532,7 +9566,7 @@
         <v>2</v>
       </c>
       <c r="C75" s="28" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="76" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9540,7 +9574,7 @@
         <v>3</v>
       </c>
       <c r="C76" s="28" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="77" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -9549,7 +9583,10 @@
         <v>447</v>
       </c>
       <c r="C78" s="62" t="s">
-        <v>522</v>
+        <v>521</v>
+      </c>
+      <c r="G78" s="27" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="79" spans="2:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9577,10 +9614,10 @@
         <v>1</v>
       </c>
       <c r="C80" s="28" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="D80" s="29" t="s">
-        <v>180</v>
+        <v>550</v>
       </c>
       <c r="E80" s="28" t="s">
         <v>200</v>
@@ -9589,7 +9626,7 @@
         <v>123456789</v>
       </c>
       <c r="G80" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="81" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9597,10 +9634,10 @@
         <v>2</v>
       </c>
       <c r="C81" s="28" t="s">
-        <v>513</v>
-      </c>
-      <c r="D81" s="28" t="s">
-        <v>181</v>
+        <v>512</v>
+      </c>
+      <c r="D81" s="66" t="s">
+        <v>551</v>
       </c>
       <c r="E81" s="28" t="s">
         <v>201</v>
@@ -9609,7 +9646,7 @@
         <v>123456789</v>
       </c>
       <c r="G81" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="82" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9617,7 +9654,7 @@
         <v>3</v>
       </c>
       <c r="C82" s="28" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D82" s="28" t="s">
         <v>182</v>
@@ -9629,7 +9666,7 @@
         <v>123456789</v>
       </c>
       <c r="G82" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="83" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9637,7 +9674,7 @@
         <v>4</v>
       </c>
       <c r="C83" s="28" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="D83" s="28" t="s">
         <v>183</v>
@@ -9649,7 +9686,7 @@
         <v>123456789</v>
       </c>
       <c r="G83" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="84" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9657,7 +9694,7 @@
         <v>5</v>
       </c>
       <c r="C84" s="28" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D84" s="28" t="s">
         <v>184</v>
@@ -9669,7 +9706,7 @@
         <v>123456789</v>
       </c>
       <c r="G84" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="85" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9677,7 +9714,7 @@
         <v>6</v>
       </c>
       <c r="C85" s="28" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D85" s="28" t="s">
         <v>185</v>
@@ -9689,7 +9726,7 @@
         <v>123456789</v>
       </c>
       <c r="G85" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="86" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9697,7 +9734,7 @@
         <v>7</v>
       </c>
       <c r="C86" s="28" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D86" s="28" t="s">
         <v>186</v>
@@ -9709,7 +9746,7 @@
         <v>123456789</v>
       </c>
       <c r="G86" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="87" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9717,7 +9754,7 @@
         <v>8</v>
       </c>
       <c r="C87" s="28" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D87" s="28" t="s">
         <v>187</v>
@@ -9729,7 +9766,7 @@
         <v>123456789</v>
       </c>
       <c r="G87" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="88" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9737,7 +9774,7 @@
         <v>9</v>
       </c>
       <c r="C88" s="28" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D88" s="28" t="s">
         <v>188</v>
@@ -9749,7 +9786,7 @@
         <v>123456789</v>
       </c>
       <c r="G88" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="89" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9757,7 +9794,7 @@
         <v>10</v>
       </c>
       <c r="C89" s="28" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D89" s="28" t="s">
         <v>189</v>
@@ -9769,13 +9806,13 @@
         <v>123456789</v>
       </c>
       <c r="G89" s="30" t="s">
-        <v>220</v>
+        <v>552</v>
       </c>
     </row>
     <row r="90" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="91" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B91" s="2" t="s">
-        <v>433</v>
+        <v>556</v>
       </c>
     </row>
     <row r="92" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -9792,7 +9829,7 @@
         <v>436</v>
       </c>
       <c r="F92" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>441</v>
@@ -9803,51 +9840,51 @@
     </row>
     <row r="93" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B93" s="28" t="s">
+        <v>522</v>
+      </c>
+      <c r="C93" s="28" t="s">
         <v>523</v>
-      </c>
-      <c r="C93" s="28" t="s">
-        <v>524</v>
       </c>
       <c r="D93" s="28">
         <v>258369741</v>
       </c>
       <c r="E93" s="28" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F93" s="28" t="s">
+        <v>526</v>
+      </c>
+      <c r="G93" s="28" t="s">
         <v>527</v>
       </c>
-      <c r="G93" s="28" t="s">
+      <c r="H93" s="28" t="s">
         <v>528</v>
-      </c>
-      <c r="H93" s="28" t="s">
-        <v>529</v>
       </c>
     </row>
     <row r="94" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B94" s="28"/>
       <c r="C94" s="28" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D94" s="28"/>
       <c r="E94" s="28"/>
       <c r="F94" s="28"/>
       <c r="G94" s="28"/>
       <c r="H94" s="28" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="95" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B95" s="28"/>
       <c r="C95" s="28" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D95" s="28"/>
       <c r="E95" s="28"/>
       <c r="F95" s="28"/>
       <c r="G95" s="28"/>
       <c r="H95" s="28" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="96" spans="2:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -9868,21 +9905,21 @@
       </c>
     </row>
     <row r="99" spans="2:4" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="71" t="s">
+      <c r="B99" s="72" t="s">
         <v>281</v>
       </c>
-      <c r="C99" s="71"/>
-      <c r="D99" s="71"/>
+      <c r="C99" s="72"/>
+      <c r="D99" s="72"/>
     </row>
     <row r="100" spans="2:4" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="71"/>
-      <c r="C100" s="71"/>
-      <c r="D100" s="71"/>
+      <c r="B100" s="72"/>
+      <c r="C100" s="72"/>
+      <c r="D100" s="72"/>
     </row>
     <row r="101" spans="2:4" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B101" s="71"/>
-      <c r="C101" s="71"/>
-      <c r="D101" s="71"/>
+      <c r="B101" s="72"/>
+      <c r="C101" s="72"/>
+      <c r="D101" s="72"/>
     </row>
     <row r="102" spans="2:4" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B102" s="28">
@@ -10442,7 +10479,7 @@
     </row>
     <row r="154" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B154" s="38" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C154" s="3" t="s">
         <v>458</v>
@@ -10454,7 +10491,7 @@
         <v>460</v>
       </c>
       <c r="F154" s="3" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="155" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -10469,7 +10506,7 @@
         <v>253</v>
       </c>
       <c r="F155" s="28" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="156" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -10501,7 +10538,7 @@
     <row r="158" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B158" s="28"/>
       <c r="C158" s="65" t="s">
-        <v>282</v>
+        <v>555</v>
       </c>
       <c r="D158" s="28"/>
       <c r="E158" s="28" t="s">
@@ -10514,7 +10551,7 @@
     <row r="159" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B159" s="28"/>
       <c r="C159" s="65" t="s">
-        <v>301</v>
+        <v>554</v>
       </c>
       <c r="D159" s="28"/>
       <c r="E159" s="28" t="s">
@@ -10544,10 +10581,10 @@
     </row>
     <row r="163" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="164" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C164" s="71" t="s">
-        <v>541</v>
-      </c>
-      <c r="D164" s="71"/>
+      <c r="C164" s="72" t="s">
+        <v>540</v>
+      </c>
+      <c r="D164" s="72"/>
     </row>
     <row r="165" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="166" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -10560,10 +10597,10 @@
     </row>
     <row r="167" spans="2:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B167" s="38" t="s">
+        <v>541</v>
+      </c>
+      <c r="C167" s="3" t="s">
         <v>542</v>
-      </c>
-      <c r="C167" s="3" t="s">
-        <v>543</v>
       </c>
       <c r="E167" s="38" t="s">
         <v>467</v>
@@ -10666,16 +10703,16 @@
         <v>476</v>
       </c>
       <c r="D177" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="E177" s="3" t="s">
         <v>544</v>
       </c>
-      <c r="E177" s="3" t="s">
+      <c r="F177" s="3" t="s">
         <v>545</v>
       </c>
-      <c r="F177" s="3" t="s">
+      <c r="G177" s="3" t="s">
         <v>546</v>
-      </c>
-      <c r="G177" s="3" t="s">
-        <v>547</v>
       </c>
       <c r="H177" s="4" t="s">
         <v>477</v>
@@ -11268,8 +11305,12 @@
     <mergeCell ref="C164:D164"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D81" r:id="rId1" xr:uid="{67FA1002-2CFA-449B-AE83-A53BB26EB143}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -12358,29 +12399,29 @@
     </row>
     <row r="33" spans="5:8" x14ac:dyDescent="0.3">
       <c r="E33" s="39" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F33" s="39"/>
     </row>
     <row r="34" spans="5:8" x14ac:dyDescent="0.3">
       <c r="E34" s="50" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="35" spans="5:8" x14ac:dyDescent="0.3">
       <c r="E35" s="50" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
     </row>
     <row r="36" spans="5:8" x14ac:dyDescent="0.3">
       <c r="E36" s="63" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="H36" s="39"/>
     </row>
     <row r="37" spans="5:8" x14ac:dyDescent="0.3">
       <c r="E37" s="50" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
   </sheetData>

</xml_diff>